<commit_message>
Update Login Test Scenario
</commit_message>
<xml_diff>
--- a/03_Test_Scenario/TestScenario_Login.xlsx
+++ b/03_Test_Scenario/TestScenario_Login.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Manual-Tester-Portfolio\03_Test_Scenario\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FBFDF7C-BA40-45AF-BDBF-A3E0D5E40D5D}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39B25B86-77E6-4C6E-B7AE-BA6740EEEAD7}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8F7A0EB9-5408-478B-92A5-4C62A1CFF411}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="47">
   <si>
     <t>Scenario ID</t>
   </si>
@@ -162,12 +162,6 @@
     <t>SC_LOGIN_013</t>
   </si>
   <si>
-    <t>Chọn Forgot Password</t>
-  </si>
-  <si>
-    <t>BR10</t>
-  </si>
-  <si>
     <t>SC_LOGIN_014</t>
   </si>
   <si>
@@ -175,9 +169,6 @@
   </si>
   <si>
     <t>BR05</t>
-  </si>
-  <si>
-    <t>SC_LOGIN_015</t>
   </si>
   <si>
     <t>Dashboard hiển thị đúng tên sinh viên sau khi Login</t>
@@ -263,42 +254,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="10">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF7D7D"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="3">
     <dxf>
       <fill>
         <patternFill>
@@ -316,21 +272,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFF7D7D"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF7D7D"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF7D7D"/>
+          <bgColor theme="9" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
@@ -649,7 +591,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23A1E97A-05AA-4A13-A2E5-86183C2B7F67}">
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.44140625" customWidth="1"/>
@@ -888,18 +830,18 @@
         <v>8</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>8</v>
@@ -914,37 +856,20 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>5</v>
-      </c>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="E2:E16">
-    <cfRule type="containsText" dxfId="5" priority="3" operator="containsText" text="High">
-      <formula>NOT(ISERROR(SEARCH("High",E2)))</formula>
+  <conditionalFormatting sqref="E2:E15">
+    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="Low">
+      <formula>NOT(ISERROR(SEARCH("Low",E2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="Medium">
+    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Medium">
       <formula>NOT(ISERROR(SEARCH("Medium",E2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Low">
-      <formula>NOT(ISERROR(SEARCH("Low",E2)))</formula>
+    <cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="High">
+      <formula>NOT(ISERROR(SEARCH("High",E2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E16" xr:uid="{335705A3-99EE-4CD4-AB69-D55C91FB5FB1}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E15" xr:uid="{335705A3-99EE-4CD4-AB69-D55C91FB5FB1}">
       <formula1>"High, Medium, Low"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>